<commit_message>
update to the authoring tool
</commit_message>
<xml_diff>
--- a/authoring/kobotoolbox/current/gaia_metadata_authoring_form_v2.xlsx
+++ b/authoring/kobotoolbox/current/gaia_metadata_authoring_form_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/davidamadi/Documents/Projects/ohdsi-gis-metadata-template/authoring/kobotoolbox/current/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1DE2B01F-AB64-854E-9A00-16783BB21412}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA524682-AE34-C849-8597-B8A0FF8492AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="2020" windowWidth="30240" windowHeight="17840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1960" uniqueCount="1047">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1961" uniqueCount="1047">
   <si>
     <t>type</t>
   </si>
@@ -3385,7 +3385,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -3501,6 +3501,7 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3667,8 +3668,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K186"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <dimension ref="A1:K187"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -7623,6 +7624,11 @@
       <c r="J186" s="16"/>
       <c r="K186" s="17"/>
     </row>
+    <row r="187" spans="1:11">
+      <c r="A187" s="43" t="s">
+        <v>37</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -7631,7 +7637,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:K197"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="36" customWidth="1"/>
@@ -7657,7 +7663,7 @@
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
     </row>
-    <row r="2" spans="1:11" ht="15">
+    <row r="2" spans="1:11">
       <c r="A2" s="36" t="s">
         <v>546</v>
       </c>
@@ -7668,7 +7674,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="15">
+    <row r="3" spans="1:11">
       <c r="A3" s="36" t="s">
         <v>546</v>
       </c>
@@ -7679,7 +7685,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="15">
+    <row r="4" spans="1:11">
       <c r="A4" s="36" t="s">
         <v>551</v>
       </c>
@@ -7690,7 +7696,7 @@
         <v>553</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="15">
+    <row r="5" spans="1:11">
       <c r="A5" s="36" t="s">
         <v>551</v>
       </c>
@@ -7701,7 +7707,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="15">
+    <row r="6" spans="1:11">
       <c r="A6" s="36" t="s">
         <v>551</v>
       </c>
@@ -7712,7 +7718,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="15">
+    <row r="7" spans="1:11">
       <c r="A7" s="36" t="s">
         <v>551</v>
       </c>
@@ -7723,7 +7729,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="15">
+    <row r="8" spans="1:11">
       <c r="A8" s="36" t="s">
         <v>551</v>
       </c>
@@ -7734,7 +7740,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="15">
+    <row r="9" spans="1:11">
       <c r="A9" s="36" t="s">
         <v>551</v>
       </c>
@@ -7745,7 +7751,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="15">
+    <row r="10" spans="1:11">
       <c r="A10" s="36" t="s">
         <v>560</v>
       </c>
@@ -7756,7 +7762,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="15">
+    <row r="11" spans="1:11">
       <c r="A11" s="36" t="s">
         <v>560</v>
       </c>
@@ -7767,7 +7773,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="15">
+    <row r="12" spans="1:11">
       <c r="A12" s="36" t="s">
         <v>560</v>
       </c>
@@ -7778,7 +7784,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="15">
+    <row r="13" spans="1:11">
       <c r="A13" s="36" t="s">
         <v>560</v>
       </c>
@@ -7789,7 +7795,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="15">
+    <row r="14" spans="1:11">
       <c r="A14" s="36" t="s">
         <v>560</v>
       </c>
@@ -7800,7 +7806,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="15">
+    <row r="15" spans="1:11">
       <c r="A15" s="36" t="s">
         <v>560</v>
       </c>
@@ -7811,7 +7817,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="15">
+    <row r="16" spans="1:11">
       <c r="A16" s="36" t="s">
         <v>560</v>
       </c>
@@ -7822,7 +7828,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15">
+    <row r="17" spans="1:3">
       <c r="A17" s="36" t="s">
         <v>574</v>
       </c>
@@ -7833,7 +7839,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="15">
+    <row r="18" spans="1:3">
       <c r="A18" s="36" t="s">
         <v>574</v>
       </c>
@@ -7844,7 +7850,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="15">
+    <row r="19" spans="1:3">
       <c r="A19" s="36" t="s">
         <v>574</v>
       </c>
@@ -7855,7 +7861,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="15">
+    <row r="20" spans="1:3">
       <c r="A20" s="36" t="s">
         <v>574</v>
       </c>
@@ -7866,7 +7872,7 @@
         <v>582</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="15">
+    <row r="21" spans="1:3">
       <c r="A21" s="36" t="s">
         <v>574</v>
       </c>
@@ -7877,7 +7883,7 @@
         <v>584</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="15">
+    <row r="22" spans="1:3">
       <c r="A22" s="36" t="s">
         <v>574</v>
       </c>
@@ -7888,7 +7894,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="15">
+    <row r="23" spans="1:3">
       <c r="A23" s="36" t="s">
         <v>574</v>
       </c>
@@ -7899,7 +7905,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="15">
+    <row r="24" spans="1:3">
       <c r="A24" s="36" t="s">
         <v>587</v>
       </c>
@@ -7910,7 +7916,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="15">
+    <row r="25" spans="1:3">
       <c r="A25" s="36" t="s">
         <v>587</v>
       </c>
@@ -7921,7 +7927,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="15">
+    <row r="26" spans="1:3">
       <c r="A26" s="36" t="s">
         <v>587</v>
       </c>
@@ -7932,7 +7938,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="15">
+    <row r="27" spans="1:3">
       <c r="A27" s="36" t="s">
         <v>587</v>
       </c>
@@ -7943,7 +7949,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="15">
+    <row r="28" spans="1:3">
       <c r="A28" s="36" t="s">
         <v>587</v>
       </c>
@@ -7954,7 +7960,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="15">
+    <row r="29" spans="1:3">
       <c r="A29" s="36" t="s">
         <v>587</v>
       </c>
@@ -7965,7 +7971,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="15">
+    <row r="30" spans="1:3">
       <c r="A30" s="36" t="s">
         <v>587</v>
       </c>
@@ -7976,7 +7982,7 @@
         <v>601</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="15">
+    <row r="31" spans="1:3">
       <c r="A31" s="36" t="s">
         <v>587</v>
       </c>
@@ -7987,7 +7993,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="15">
+    <row r="32" spans="1:3">
       <c r="A32" s="36" t="s">
         <v>604</v>
       </c>
@@ -7998,7 +8004,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="15">
+    <row r="33" spans="1:3">
       <c r="A33" s="36" t="s">
         <v>604</v>
       </c>
@@ -8009,7 +8015,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="15">
+    <row r="34" spans="1:3">
       <c r="A34" s="36" t="s">
         <v>604</v>
       </c>
@@ -8020,7 +8026,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="15">
+    <row r="35" spans="1:3">
       <c r="A35" s="36" t="s">
         <v>604</v>
       </c>
@@ -8031,7 +8037,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="36" spans="1:3" ht="15">
+    <row r="36" spans="1:3">
       <c r="A36" s="36" t="s">
         <v>604</v>
       </c>
@@ -8042,7 +8048,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="15">
+    <row r="37" spans="1:3">
       <c r="A37" s="36" t="s">
         <v>613</v>
       </c>
@@ -8053,7 +8059,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ht="15">
+    <row r="38" spans="1:3">
       <c r="A38" s="36" t="s">
         <v>613</v>
       </c>
@@ -8064,7 +8070,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="15">
+    <row r="39" spans="1:3">
       <c r="A39" s="36" t="s">
         <v>613</v>
       </c>
@@ -8075,7 +8081,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ht="15">
+    <row r="40" spans="1:3">
       <c r="A40" s="36" t="s">
         <v>613</v>
       </c>
@@ -8086,7 +8092,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="41" spans="1:3" ht="15">
+    <row r="41" spans="1:3">
       <c r="A41" s="36" t="s">
         <v>613</v>
       </c>
@@ -8097,7 +8103,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ht="15">
+    <row r="42" spans="1:3">
       <c r="A42" s="36" t="s">
         <v>613</v>
       </c>
@@ -8108,7 +8114,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="43" spans="1:3" ht="15">
+    <row r="43" spans="1:3">
       <c r="A43" s="36" t="s">
         <v>617</v>
       </c>
@@ -8119,7 +8125,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="15">
+    <row r="44" spans="1:3">
       <c r="A44" s="36" t="s">
         <v>617</v>
       </c>
@@ -8130,7 +8136,7 @@
         <v>619</v>
       </c>
     </row>
-    <row r="45" spans="1:3" ht="15">
+    <row r="45" spans="1:3">
       <c r="A45" s="36" t="s">
         <v>617</v>
       </c>
@@ -8141,7 +8147,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="46" spans="1:3" ht="15">
+    <row r="46" spans="1:3">
       <c r="A46" s="36" t="s">
         <v>617</v>
       </c>
@@ -8152,7 +8158,7 @@
         <v>621</v>
       </c>
     </row>
-    <row r="47" spans="1:3" ht="15">
+    <row r="47" spans="1:3">
       <c r="A47" s="36" t="s">
         <v>617</v>
       </c>
@@ -8163,7 +8169,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="48" spans="1:3" ht="15">
+    <row r="48" spans="1:3">
       <c r="A48" s="36" t="s">
         <v>617</v>
       </c>
@@ -8174,7 +8180,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="49" spans="1:3" ht="15">
+    <row r="49" spans="1:3">
       <c r="A49" s="36" t="s">
         <v>617</v>
       </c>
@@ -8185,7 +8191,7 @@
         <v>624</v>
       </c>
     </row>
-    <row r="50" spans="1:3" ht="15">
+    <row r="50" spans="1:3">
       <c r="A50" s="36" t="s">
         <v>248</v>
       </c>
@@ -8196,7 +8202,7 @@
         <v>625</v>
       </c>
     </row>
-    <row r="51" spans="1:3" ht="15">
+    <row r="51" spans="1:3">
       <c r="A51" s="36" t="s">
         <v>248</v>
       </c>
@@ -8207,7 +8213,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="52" spans="1:3" ht="15">
+    <row r="52" spans="1:3">
       <c r="A52" s="36" t="s">
         <v>248</v>
       </c>
@@ -8218,7 +8224,7 @@
         <v>627</v>
       </c>
     </row>
-    <row r="53" spans="1:3" ht="15">
+    <row r="53" spans="1:3">
       <c r="A53" s="36" t="s">
         <v>248</v>
       </c>
@@ -8229,7 +8235,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="54" spans="1:3" ht="15">
+    <row r="54" spans="1:3">
       <c r="A54" s="36" t="s">
         <v>248</v>
       </c>
@@ -8240,7 +8246,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="55" spans="1:3" ht="15">
+    <row r="55" spans="1:3">
       <c r="A55" s="36" t="s">
         <v>629</v>
       </c>
@@ -8251,7 +8257,7 @@
         <v>631</v>
       </c>
     </row>
-    <row r="56" spans="1:3" ht="15">
+    <row r="56" spans="1:3">
       <c r="A56" s="36" t="s">
         <v>629</v>
       </c>
@@ -8262,7 +8268,7 @@
         <v>633</v>
       </c>
     </row>
-    <row r="57" spans="1:3" ht="15">
+    <row r="57" spans="1:3">
       <c r="A57" s="36" t="s">
         <v>629</v>
       </c>
@@ -8273,7 +8279,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="58" spans="1:3" ht="15">
+    <row r="58" spans="1:3">
       <c r="A58" s="36" t="s">
         <v>629</v>
       </c>
@@ -8284,7 +8290,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="59" spans="1:3" ht="15">
+    <row r="59" spans="1:3">
       <c r="A59" s="36" t="s">
         <v>629</v>
       </c>
@@ -8295,7 +8301,7 @@
         <v>639</v>
       </c>
     </row>
-    <row r="60" spans="1:3" ht="15">
+    <row r="60" spans="1:3">
       <c r="A60" s="36" t="s">
         <v>629</v>
       </c>
@@ -8306,7 +8312,7 @@
         <v>641</v>
       </c>
     </row>
-    <row r="61" spans="1:3" ht="15">
+    <row r="61" spans="1:3">
       <c r="A61" s="36" t="s">
         <v>629</v>
       </c>
@@ -8317,7 +8323,7 @@
         <v>643</v>
       </c>
     </row>
-    <row r="62" spans="1:3" ht="15">
+    <row r="62" spans="1:3">
       <c r="A62" s="36" t="s">
         <v>629</v>
       </c>
@@ -8328,7 +8334,7 @@
         <v>645</v>
       </c>
     </row>
-    <row r="63" spans="1:3" ht="15">
+    <row r="63" spans="1:3">
       <c r="A63" s="36" t="s">
         <v>629</v>
       </c>
@@ -8339,7 +8345,7 @@
         <v>647</v>
       </c>
     </row>
-    <row r="64" spans="1:3" ht="15">
+    <row r="64" spans="1:3">
       <c r="A64" s="36" t="s">
         <v>648</v>
       </c>
@@ -8350,7 +8356,7 @@
         <v>649</v>
       </c>
     </row>
-    <row r="65" spans="1:3" ht="15">
+    <row r="65" spans="1:3">
       <c r="A65" s="36" t="s">
         <v>648</v>
       </c>
@@ -8361,7 +8367,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="66" spans="1:3" ht="15">
+    <row r="66" spans="1:3">
       <c r="A66" s="36" t="s">
         <v>648</v>
       </c>
@@ -8372,7 +8378,7 @@
         <v>652</v>
       </c>
     </row>
-    <row r="67" spans="1:3" ht="15">
+    <row r="67" spans="1:3">
       <c r="A67" s="36" t="s">
         <v>648</v>
       </c>
@@ -8383,7 +8389,7 @@
         <v>653</v>
       </c>
     </row>
-    <row r="68" spans="1:3" ht="15">
+    <row r="68" spans="1:3">
       <c r="A68" s="36" t="s">
         <v>648</v>
       </c>
@@ -8394,7 +8400,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="69" spans="1:3" ht="15">
+    <row r="69" spans="1:3">
       <c r="A69" s="36" t="s">
         <v>654</v>
       </c>
@@ -8405,7 +8411,7 @@
         <v>655</v>
       </c>
     </row>
-    <row r="70" spans="1:3" ht="15">
+    <row r="70" spans="1:3">
       <c r="A70" s="36" t="s">
         <v>654</v>
       </c>
@@ -8416,7 +8422,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="71" spans="1:3" ht="15">
+    <row r="71" spans="1:3">
       <c r="A71" s="36" t="s">
         <v>654</v>
       </c>
@@ -8427,7 +8433,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="72" spans="1:3" ht="15">
+    <row r="72" spans="1:3">
       <c r="A72" s="36" t="s">
         <v>654</v>
       </c>
@@ -8438,7 +8444,7 @@
         <v>657</v>
       </c>
     </row>
-    <row r="73" spans="1:3" ht="15">
+    <row r="73" spans="1:3">
       <c r="A73" s="36" t="s">
         <v>654</v>
       </c>
@@ -8449,7 +8455,7 @@
         <v>658</v>
       </c>
     </row>
-    <row r="74" spans="1:3" ht="15">
+    <row r="74" spans="1:3">
       <c r="A74" s="36" t="s">
         <v>654</v>
       </c>
@@ -8460,7 +8466,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="75" spans="1:3" ht="15">
+    <row r="75" spans="1:3">
       <c r="A75" s="36" t="s">
         <v>654</v>
       </c>
@@ -8471,7 +8477,7 @@
         <v>659</v>
       </c>
     </row>
-    <row r="76" spans="1:3" ht="15">
+    <row r="76" spans="1:3">
       <c r="A76" s="36" t="s">
         <v>654</v>
       </c>
@@ -8482,7 +8488,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="77" spans="1:3" ht="15">
+    <row r="77" spans="1:3">
       <c r="A77" s="36" t="s">
         <v>654</v>
       </c>
@@ -8493,7 +8499,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="78" spans="1:3" ht="15">
+    <row r="78" spans="1:3">
       <c r="A78" s="36" t="s">
         <v>660</v>
       </c>
@@ -8504,7 +8510,7 @@
         <v>661</v>
       </c>
     </row>
-    <row r="79" spans="1:3" ht="15">
+    <row r="79" spans="1:3">
       <c r="A79" s="36" t="s">
         <v>660</v>
       </c>
@@ -8515,7 +8521,7 @@
         <v>662</v>
       </c>
     </row>
-    <row r="80" spans="1:3" ht="15">
+    <row r="80" spans="1:3">
       <c r="A80" s="36" t="s">
         <v>660</v>
       </c>
@@ -8526,7 +8532,7 @@
         <v>663</v>
       </c>
     </row>
-    <row r="81" spans="1:3" ht="15">
+    <row r="81" spans="1:3">
       <c r="A81" s="36" t="s">
         <v>398</v>
       </c>
@@ -8537,7 +8543,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="82" spans="1:3" ht="15">
+    <row r="82" spans="1:3">
       <c r="A82" s="36" t="s">
         <v>398</v>
       </c>
@@ -8548,7 +8554,7 @@
         <v>667</v>
       </c>
     </row>
-    <row r="83" spans="1:3" ht="15">
+    <row r="83" spans="1:3">
       <c r="A83" s="36" t="s">
         <v>398</v>
       </c>
@@ -8559,7 +8565,7 @@
         <v>669</v>
       </c>
     </row>
-    <row r="84" spans="1:3" ht="15">
+    <row r="84" spans="1:3">
       <c r="A84" s="36" t="s">
         <v>398</v>
       </c>
@@ -8570,7 +8576,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="85" spans="1:3" ht="15">
+    <row r="85" spans="1:3">
       <c r="A85" s="36" t="s">
         <v>398</v>
       </c>
@@ -8581,7 +8587,7 @@
         <v>673</v>
       </c>
     </row>
-    <row r="86" spans="1:3" ht="15">
+    <row r="86" spans="1:3">
       <c r="A86" s="36" t="s">
         <v>398</v>
       </c>
@@ -8592,7 +8598,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="87" spans="1:3" ht="15">
+    <row r="87" spans="1:3">
       <c r="A87" s="36" t="s">
         <v>398</v>
       </c>
@@ -8603,7 +8609,7 @@
         <v>677</v>
       </c>
     </row>
-    <row r="88" spans="1:3" ht="15">
+    <row r="88" spans="1:3">
       <c r="A88" s="36" t="s">
         <v>398</v>
       </c>
@@ -8614,7 +8620,7 @@
         <v>679</v>
       </c>
     </row>
-    <row r="89" spans="1:3" ht="15">
+    <row r="89" spans="1:3">
       <c r="A89" s="36" t="s">
         <v>398</v>
       </c>
@@ -8625,7 +8631,7 @@
         <v>681</v>
       </c>
     </row>
-    <row r="90" spans="1:3" ht="15">
+    <row r="90" spans="1:3">
       <c r="A90" s="36" t="s">
         <v>398</v>
       </c>
@@ -8636,7 +8642,7 @@
         <v>683</v>
       </c>
     </row>
-    <row r="91" spans="1:3" ht="15">
+    <row r="91" spans="1:3">
       <c r="A91" s="36" t="s">
         <v>398</v>
       </c>
@@ -8647,7 +8653,7 @@
         <v>685</v>
       </c>
     </row>
-    <row r="92" spans="1:3" ht="15">
+    <row r="92" spans="1:3">
       <c r="A92" s="36" t="s">
         <v>398</v>
       </c>
@@ -8658,7 +8664,7 @@
         <v>687</v>
       </c>
     </row>
-    <row r="93" spans="1:3" ht="15">
+    <row r="93" spans="1:3">
       <c r="A93" s="36" t="s">
         <v>398</v>
       </c>
@@ -8669,7 +8675,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="94" spans="1:3" ht="15">
+    <row r="94" spans="1:3">
       <c r="A94" s="36" t="s">
         <v>398</v>
       </c>
@@ -8680,7 +8686,7 @@
         <v>691</v>
       </c>
     </row>
-    <row r="95" spans="1:3" ht="15">
+    <row r="95" spans="1:3">
       <c r="A95" s="36" t="s">
         <v>398</v>
       </c>
@@ -8691,7 +8697,7 @@
         <v>693</v>
       </c>
     </row>
-    <row r="96" spans="1:3" ht="15">
+    <row r="96" spans="1:3">
       <c r="A96" s="36" t="s">
         <v>398</v>
       </c>
@@ -8702,7 +8708,7 @@
         <v>695</v>
       </c>
     </row>
-    <row r="97" spans="1:3" ht="15">
+    <row r="97" spans="1:3">
       <c r="A97" s="36" t="s">
         <v>398</v>
       </c>
@@ -8713,7 +8719,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="98" spans="1:3" ht="15">
+    <row r="98" spans="1:3">
       <c r="A98" s="36" t="s">
         <v>398</v>
       </c>
@@ -8724,7 +8730,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="99" spans="1:3" ht="15">
+    <row r="99" spans="1:3">
       <c r="A99" s="36" t="s">
         <v>398</v>
       </c>
@@ -8735,7 +8741,7 @@
         <v>701</v>
       </c>
     </row>
-    <row r="100" spans="1:3" ht="15">
+    <row r="100" spans="1:3">
       <c r="A100" s="36" t="s">
         <v>398</v>
       </c>
@@ -8746,7 +8752,7 @@
         <v>703</v>
       </c>
     </row>
-    <row r="101" spans="1:3" ht="15">
+    <row r="101" spans="1:3">
       <c r="A101" s="36" t="s">
         <v>398</v>
       </c>
@@ -8757,7 +8763,7 @@
         <v>705</v>
       </c>
     </row>
-    <row r="102" spans="1:3" ht="15">
+    <row r="102" spans="1:3">
       <c r="A102" s="36" t="s">
         <v>398</v>
       </c>
@@ -8768,7 +8774,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="103" spans="1:3" ht="15">
+    <row r="103" spans="1:3">
       <c r="A103" s="36" t="s">
         <v>398</v>
       </c>
@@ -8779,7 +8785,7 @@
         <v>709</v>
       </c>
     </row>
-    <row r="104" spans="1:3" ht="15">
+    <row r="104" spans="1:3">
       <c r="A104" s="36" t="s">
         <v>398</v>
       </c>
@@ -8790,7 +8796,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="105" spans="1:3" ht="15">
+    <row r="105" spans="1:3">
       <c r="A105" s="36" t="s">
         <v>398</v>
       </c>
@@ -8801,7 +8807,7 @@
         <v>713</v>
       </c>
     </row>
-    <row r="106" spans="1:3" ht="15">
+    <row r="106" spans="1:3">
       <c r="A106" s="36" t="s">
         <v>398</v>
       </c>
@@ -8812,7 +8818,7 @@
         <v>715</v>
       </c>
     </row>
-    <row r="107" spans="1:3" ht="15">
+    <row r="107" spans="1:3">
       <c r="A107" s="36" t="s">
         <v>398</v>
       </c>
@@ -8823,7 +8829,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="108" spans="1:3" ht="15">
+    <row r="108" spans="1:3">
       <c r="A108" s="36" t="s">
         <v>398</v>
       </c>
@@ -8834,7 +8840,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="109" spans="1:3" ht="15">
+    <row r="109" spans="1:3">
       <c r="A109" s="36" t="s">
         <v>398</v>
       </c>
@@ -8845,7 +8851,7 @@
         <v>721</v>
       </c>
     </row>
-    <row r="110" spans="1:3" ht="15">
+    <row r="110" spans="1:3">
       <c r="A110" s="36" t="s">
         <v>398</v>
       </c>
@@ -8856,7 +8862,7 @@
         <v>723</v>
       </c>
     </row>
-    <row r="111" spans="1:3" ht="15">
+    <row r="111" spans="1:3">
       <c r="A111" s="36" t="s">
         <v>398</v>
       </c>
@@ -8867,7 +8873,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="112" spans="1:3" ht="15">
+    <row r="112" spans="1:3">
       <c r="A112" s="36" t="s">
         <v>398</v>
       </c>
@@ -8878,7 +8884,7 @@
         <v>727</v>
       </c>
     </row>
-    <row r="113" spans="1:3" ht="15">
+    <row r="113" spans="1:3">
       <c r="A113" s="36" t="s">
         <v>728</v>
       </c>
@@ -8889,7 +8895,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="114" spans="1:3" ht="15">
+    <row r="114" spans="1:3">
       <c r="A114" s="36" t="s">
         <v>728</v>
       </c>
@@ -8900,7 +8906,7 @@
         <v>732</v>
       </c>
     </row>
-    <row r="115" spans="1:3" ht="15">
+    <row r="115" spans="1:3">
       <c r="A115" s="36" t="s">
         <v>728</v>
       </c>
@@ -8911,7 +8917,7 @@
         <v>734</v>
       </c>
     </row>
-    <row r="116" spans="1:3" ht="15">
+    <row r="116" spans="1:3">
       <c r="A116" s="36" t="s">
         <v>728</v>
       </c>
@@ -8922,7 +8928,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="117" spans="1:3" ht="15">
+    <row r="117" spans="1:3">
       <c r="A117" s="36" t="s">
         <v>728</v>
       </c>
@@ -8933,7 +8939,7 @@
         <v>738</v>
       </c>
     </row>
-    <row r="118" spans="1:3" ht="15">
+    <row r="118" spans="1:3">
       <c r="A118" s="36" t="s">
         <v>728</v>
       </c>
@@ -8944,7 +8950,7 @@
         <v>740</v>
       </c>
     </row>
-    <row r="119" spans="1:3" ht="15">
+    <row r="119" spans="1:3">
       <c r="A119" s="36" t="s">
         <v>728</v>
       </c>
@@ -8955,7 +8961,7 @@
         <v>631</v>
       </c>
     </row>
-    <row r="120" spans="1:3" ht="15">
+    <row r="120" spans="1:3">
       <c r="A120" s="36" t="s">
         <v>741</v>
       </c>
@@ -8966,7 +8972,7 @@
         <v>631</v>
       </c>
     </row>
-    <row r="121" spans="1:3" ht="15">
+    <row r="121" spans="1:3">
       <c r="A121" s="36" t="s">
         <v>741</v>
       </c>
@@ -8977,7 +8983,7 @@
         <v>743</v>
       </c>
     </row>
-    <row r="122" spans="1:3" ht="15">
+    <row r="122" spans="1:3">
       <c r="A122" s="36" t="s">
         <v>741</v>
       </c>
@@ -8988,7 +8994,7 @@
         <v>745</v>
       </c>
     </row>
-    <row r="123" spans="1:3" ht="15">
+    <row r="123" spans="1:3">
       <c r="A123" s="36" t="s">
         <v>741</v>
       </c>
@@ -8999,7 +9005,7 @@
         <v>747</v>
       </c>
     </row>
-    <row r="124" spans="1:3" ht="15">
+    <row r="124" spans="1:3">
       <c r="A124" s="36" t="s">
         <v>741</v>
       </c>
@@ -9010,7 +9016,7 @@
         <v>749</v>
       </c>
     </row>
-    <row r="125" spans="1:3" ht="15">
+    <row r="125" spans="1:3">
       <c r="A125" s="36" t="s">
         <v>741</v>
       </c>
@@ -9021,7 +9027,7 @@
         <v>751</v>
       </c>
     </row>
-    <row r="126" spans="1:3" ht="15">
+    <row r="126" spans="1:3">
       <c r="A126" s="36" t="s">
         <v>752</v>
       </c>
@@ -9032,7 +9038,7 @@
         <v>754</v>
       </c>
     </row>
-    <row r="127" spans="1:3" ht="15">
+    <row r="127" spans="1:3">
       <c r="A127" s="36" t="s">
         <v>752</v>
       </c>
@@ -9043,7 +9049,7 @@
         <v>755</v>
       </c>
     </row>
-    <row r="128" spans="1:3" ht="15">
+    <row r="128" spans="1:3">
       <c r="A128" s="36" t="s">
         <v>752</v>
       </c>
@@ -9054,7 +9060,7 @@
         <v>757</v>
       </c>
     </row>
-    <row r="129" spans="1:3" ht="15">
+    <row r="129" spans="1:3">
       <c r="A129" s="36" t="s">
         <v>758</v>
       </c>
@@ -9065,7 +9071,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="130" spans="1:3" ht="15">
+    <row r="130" spans="1:3">
       <c r="A130" s="36" t="s">
         <v>758</v>
       </c>
@@ -9076,7 +9082,7 @@
         <v>760</v>
       </c>
     </row>
-    <row r="131" spans="1:3" ht="15">
+    <row r="131" spans="1:3">
       <c r="A131" s="36" t="s">
         <v>758</v>
       </c>
@@ -9087,7 +9093,7 @@
         <v>762</v>
       </c>
     </row>
-    <row r="132" spans="1:3" ht="15">
+    <row r="132" spans="1:3">
       <c r="A132" s="36" t="s">
         <v>758</v>
       </c>
@@ -9098,7 +9104,7 @@
         <v>764</v>
       </c>
     </row>
-    <row r="133" spans="1:3" ht="15">
+    <row r="133" spans="1:3">
       <c r="A133" s="36" t="s">
         <v>758</v>
       </c>
@@ -9109,7 +9115,7 @@
         <v>766</v>
       </c>
     </row>
-    <row r="134" spans="1:3" ht="15">
+    <row r="134" spans="1:3">
       <c r="A134" s="36" t="s">
         <v>758</v>
       </c>
@@ -9120,7 +9126,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="135" spans="1:3" ht="15">
+    <row r="135" spans="1:3">
       <c r="A135" s="36" t="s">
         <v>758</v>
       </c>
@@ -9131,7 +9137,7 @@
         <v>768</v>
       </c>
     </row>
-    <row r="136" spans="1:3" ht="15">
+    <row r="136" spans="1:3">
       <c r="A136" s="36" t="s">
         <v>758</v>
       </c>
@@ -9142,7 +9148,7 @@
         <v>769</v>
       </c>
     </row>
-    <row r="137" spans="1:3" ht="15">
+    <row r="137" spans="1:3">
       <c r="A137" s="36" t="s">
         <v>758</v>
       </c>
@@ -9153,7 +9159,7 @@
         <v>771</v>
       </c>
     </row>
-    <row r="138" spans="1:3" ht="15">
+    <row r="138" spans="1:3">
       <c r="A138" s="36" t="s">
         <v>758</v>
       </c>
@@ -9164,7 +9170,7 @@
         <v>772</v>
       </c>
     </row>
-    <row r="139" spans="1:3" ht="15">
+    <row r="139" spans="1:3">
       <c r="A139" s="36" t="s">
         <v>758</v>
       </c>
@@ -9175,7 +9181,7 @@
         <v>774</v>
       </c>
     </row>
-    <row r="140" spans="1:3" ht="15">
+    <row r="140" spans="1:3">
       <c r="A140" s="36" t="s">
         <v>758</v>
       </c>
@@ -9186,7 +9192,7 @@
         <v>776</v>
       </c>
     </row>
-    <row r="141" spans="1:3" ht="15">
+    <row r="141" spans="1:3">
       <c r="A141" s="36" t="s">
         <v>758</v>
       </c>
@@ -9197,7 +9203,7 @@
         <v>778</v>
       </c>
     </row>
-    <row r="142" spans="1:3" ht="15">
+    <row r="142" spans="1:3">
       <c r="A142" s="36" t="s">
         <v>758</v>
       </c>
@@ -9208,7 +9214,7 @@
         <v>780</v>
       </c>
     </row>
-    <row r="143" spans="1:3" ht="15">
+    <row r="143" spans="1:3">
       <c r="A143" s="36" t="s">
         <v>758</v>
       </c>
@@ -9219,7 +9225,7 @@
         <v>631</v>
       </c>
     </row>
-    <row r="144" spans="1:3" ht="15">
+    <row r="144" spans="1:3">
       <c r="A144" s="36" t="s">
         <v>781</v>
       </c>
@@ -9230,7 +9236,7 @@
         <v>782</v>
       </c>
     </row>
-    <row r="145" spans="1:3" ht="15">
+    <row r="145" spans="1:3">
       <c r="A145" s="36" t="s">
         <v>781</v>
       </c>
@@ -9241,7 +9247,7 @@
         <v>746</v>
       </c>
     </row>
-    <row r="146" spans="1:3" ht="15">
+    <row r="146" spans="1:3">
       <c r="A146" s="36" t="s">
         <v>781</v>
       </c>
@@ -9252,7 +9258,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="147" spans="1:3" ht="15">
+    <row r="147" spans="1:3">
       <c r="A147" s="36" t="s">
         <v>781</v>
       </c>
@@ -9263,7 +9269,7 @@
         <v>744</v>
       </c>
     </row>
-    <row r="148" spans="1:3" ht="15">
+    <row r="148" spans="1:3">
       <c r="A148" s="36" t="s">
         <v>781</v>
       </c>
@@ -9274,7 +9280,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="149" spans="1:3" ht="15">
+    <row r="149" spans="1:3">
       <c r="A149" s="36" t="s">
         <v>781</v>
       </c>
@@ -9285,7 +9291,7 @@
         <v>783</v>
       </c>
     </row>
-    <row r="150" spans="1:3" ht="15">
+    <row r="150" spans="1:3">
       <c r="A150" s="36" t="s">
         <v>781</v>
       </c>
@@ -9296,7 +9302,7 @@
         <v>784</v>
       </c>
     </row>
-    <row r="151" spans="1:3" ht="15">
+    <row r="151" spans="1:3">
       <c r="A151" s="36" t="s">
         <v>781</v>
       </c>
@@ -9307,7 +9313,7 @@
         <v>785</v>
       </c>
     </row>
-    <row r="152" spans="1:3" ht="15">
+    <row r="152" spans="1:3">
       <c r="A152" s="36" t="s">
         <v>781</v>
       </c>
@@ -9318,7 +9324,7 @@
         <v>786</v>
       </c>
     </row>
-    <row r="153" spans="1:3" ht="15">
+    <row r="153" spans="1:3">
       <c r="A153" s="36" t="s">
         <v>781</v>
       </c>
@@ -9329,7 +9335,7 @@
         <v>788</v>
       </c>
     </row>
-    <row r="154" spans="1:3" ht="15">
+    <row r="154" spans="1:3">
       <c r="A154" s="36" t="s">
         <v>781</v>
       </c>
@@ -9340,7 +9346,7 @@
         <v>789</v>
       </c>
     </row>
-    <row r="155" spans="1:3" ht="15">
+    <row r="155" spans="1:3">
       <c r="A155" s="36" t="s">
         <v>781</v>
       </c>
@@ -9351,7 +9357,7 @@
         <v>790</v>
       </c>
     </row>
-    <row r="156" spans="1:3" ht="15">
+    <row r="156" spans="1:3">
       <c r="A156" s="36" t="s">
         <v>781</v>
       </c>
@@ -9362,7 +9368,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="157" spans="1:3" ht="15">
+    <row r="157" spans="1:3">
       <c r="A157" s="36" t="s">
         <v>791</v>
       </c>
@@ -9373,7 +9379,7 @@
         <v>769</v>
       </c>
     </row>
-    <row r="158" spans="1:3" ht="15">
+    <row r="158" spans="1:3">
       <c r="A158" s="36" t="s">
         <v>791</v>
       </c>
@@ -9384,7 +9390,7 @@
         <v>792</v>
       </c>
     </row>
-    <row r="159" spans="1:3" ht="15">
+    <row r="159" spans="1:3">
       <c r="A159" s="36" t="s">
         <v>791</v>
       </c>
@@ -9395,7 +9401,7 @@
         <v>772</v>
       </c>
     </row>
-    <row r="160" spans="1:3" ht="15">
+    <row r="160" spans="1:3">
       <c r="A160" s="36" t="s">
         <v>791</v>
       </c>
@@ -9406,7 +9412,7 @@
         <v>793</v>
       </c>
     </row>
-    <row r="161" spans="1:3" ht="15">
+    <row r="161" spans="1:3">
       <c r="A161" s="36" t="s">
         <v>791</v>
       </c>
@@ -9417,7 +9423,7 @@
         <v>779</v>
       </c>
     </row>
-    <row r="162" spans="1:3" ht="15">
+    <row r="162" spans="1:3">
       <c r="A162" s="36" t="s">
         <v>791</v>
       </c>
@@ -9428,7 +9434,7 @@
         <v>777</v>
       </c>
     </row>
-    <row r="163" spans="1:3" ht="15">
+    <row r="163" spans="1:3">
       <c r="A163" s="36" t="s">
         <v>791</v>
       </c>
@@ -9439,7 +9445,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="164" spans="1:3" ht="15">
+    <row r="164" spans="1:3">
       <c r="A164" s="36" t="s">
         <v>791</v>
       </c>
@@ -9450,7 +9456,7 @@
         <v>631</v>
       </c>
     </row>
-    <row r="165" spans="1:3" ht="15">
+    <row r="165" spans="1:3">
       <c r="A165" s="36" t="s">
         <v>795</v>
       </c>
@@ -9461,7 +9467,7 @@
         <v>631</v>
       </c>
     </row>
-    <row r="166" spans="1:3" ht="15">
+    <row r="166" spans="1:3">
       <c r="A166" s="36" t="s">
         <v>795</v>
       </c>
@@ -9472,7 +9478,7 @@
         <v>784</v>
       </c>
     </row>
-    <row r="167" spans="1:3" ht="15">
+    <row r="167" spans="1:3">
       <c r="A167" s="36" t="s">
         <v>795</v>
       </c>
@@ -9483,7 +9489,7 @@
         <v>746</v>
       </c>
     </row>
-    <row r="168" spans="1:3" ht="15">
+    <row r="168" spans="1:3">
       <c r="A168" s="36" t="s">
         <v>795</v>
       </c>
@@ -9494,7 +9500,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="169" spans="1:3" ht="15">
+    <row r="169" spans="1:3">
       <c r="A169" s="36" t="s">
         <v>795</v>
       </c>
@@ -9505,7 +9511,7 @@
         <v>744</v>
       </c>
     </row>
-    <row r="170" spans="1:3" ht="15">
+    <row r="170" spans="1:3">
       <c r="A170" s="36" t="s">
         <v>795</v>
       </c>
@@ -9516,7 +9522,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="171" spans="1:3" ht="15">
+    <row r="171" spans="1:3">
       <c r="A171" s="36" t="s">
         <v>795</v>
       </c>
@@ -9527,7 +9533,7 @@
         <v>783</v>
       </c>
     </row>
-    <row r="172" spans="1:3" ht="15">
+    <row r="172" spans="1:3">
       <c r="A172" s="36" t="s">
         <v>795</v>
       </c>
@@ -9538,7 +9544,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="173" spans="1:3" ht="15">
+    <row r="173" spans="1:3">
       <c r="A173" s="36" t="s">
         <v>795</v>
       </c>
@@ -9549,7 +9555,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="174" spans="1:3" ht="15">
+    <row r="174" spans="1:3">
       <c r="A174" s="36" t="s">
         <v>795</v>
       </c>
@@ -9560,7 +9566,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="175" spans="1:3" ht="15">
+    <row r="175" spans="1:3">
       <c r="A175" s="36" t="s">
         <v>795</v>
       </c>
@@ -9571,7 +9577,7 @@
         <v>796</v>
       </c>
     </row>
-    <row r="176" spans="1:3" ht="15">
+    <row r="176" spans="1:3">
       <c r="A176" s="36" t="s">
         <v>795</v>
       </c>
@@ -9582,7 +9588,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="177" spans="1:3" ht="15">
+    <row r="177" spans="1:3">
       <c r="A177" s="36" t="s">
         <v>797</v>
       </c>
@@ -9593,7 +9599,7 @@
         <v>631</v>
       </c>
     </row>
-    <row r="178" spans="1:3" ht="15">
+    <row r="178" spans="1:3">
       <c r="A178" s="36" t="s">
         <v>797</v>
       </c>
@@ -9604,7 +9610,7 @@
         <v>798</v>
       </c>
     </row>
-    <row r="179" spans="1:3" ht="15">
+    <row r="179" spans="1:3">
       <c r="A179" s="36" t="s">
         <v>797</v>
       </c>
@@ -9615,7 +9621,7 @@
         <v>799</v>
       </c>
     </row>
-    <row r="180" spans="1:3" ht="15">
+    <row r="180" spans="1:3">
       <c r="A180" s="36" t="s">
         <v>797</v>
       </c>
@@ -9626,7 +9632,7 @@
         <v>800</v>
       </c>
     </row>
-    <row r="181" spans="1:3" ht="15">
+    <row r="181" spans="1:3">
       <c r="A181" s="36" t="s">
         <v>797</v>
       </c>
@@ -9637,7 +9643,7 @@
         <v>801</v>
       </c>
     </row>
-    <row r="182" spans="1:3" ht="15">
+    <row r="182" spans="1:3">
       <c r="A182" s="36" t="s">
         <v>797</v>
       </c>
@@ -9648,7 +9654,7 @@
         <v>802</v>
       </c>
     </row>
-    <row r="183" spans="1:3" ht="15">
+    <row r="183" spans="1:3">
       <c r="A183" s="36" t="s">
         <v>797</v>
       </c>
@@ -9659,7 +9665,7 @@
         <v>803</v>
       </c>
     </row>
-    <row r="184" spans="1:3" ht="15">
+    <row r="184" spans="1:3">
       <c r="A184" s="36" t="s">
         <v>797</v>
       </c>
@@ -9670,7 +9676,7 @@
         <v>804</v>
       </c>
     </row>
-    <row r="185" spans="1:3" ht="15">
+    <row r="185" spans="1:3">
       <c r="A185" s="36" t="s">
         <v>797</v>
       </c>
@@ -9681,7 +9687,7 @@
         <v>805</v>
       </c>
     </row>
-    <row r="186" spans="1:3" ht="15">
+    <row r="186" spans="1:3">
       <c r="A186" s="36" t="s">
         <v>797</v>
       </c>
@@ -9692,7 +9698,7 @@
         <v>806</v>
       </c>
     </row>
-    <row r="187" spans="1:3" ht="15">
+    <row r="187" spans="1:3">
       <c r="A187" s="36" t="s">
         <v>807</v>
       </c>
@@ -9703,7 +9709,7 @@
         <v>808</v>
       </c>
     </row>
-    <row r="188" spans="1:3" ht="15">
+    <row r="188" spans="1:3">
       <c r="A188" s="36" t="s">
         <v>807</v>
       </c>
@@ -9714,7 +9720,7 @@
         <v>809</v>
       </c>
     </row>
-    <row r="189" spans="1:3" ht="15">
+    <row r="189" spans="1:3">
       <c r="A189" s="36" t="s">
         <v>807</v>
       </c>
@@ -9725,7 +9731,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="190" spans="1:3" ht="15">
+    <row r="190" spans="1:3">
       <c r="A190" s="36" t="s">
         <v>810</v>
       </c>
@@ -9736,7 +9742,7 @@
         <v>812</v>
       </c>
     </row>
-    <row r="191" spans="1:3" ht="15">
+    <row r="191" spans="1:3">
       <c r="A191" s="36" t="s">
         <v>810</v>
       </c>
@@ -9747,7 +9753,7 @@
         <v>814</v>
       </c>
     </row>
-    <row r="192" spans="1:3" ht="15">
+    <row r="192" spans="1:3">
       <c r="A192" s="36" t="s">
         <v>810</v>
       </c>
@@ -9758,7 +9764,7 @@
         <v>816</v>
       </c>
     </row>
-    <row r="193" spans="1:3" ht="15">
+    <row r="193" spans="1:3">
       <c r="A193" s="36" t="s">
         <v>810</v>
       </c>
@@ -9769,7 +9775,7 @@
         <v>818</v>
       </c>
     </row>
-    <row r="194" spans="1:3" ht="15">
+    <row r="194" spans="1:3">
       <c r="A194" s="36" t="s">
         <v>810</v>
       </c>
@@ -9780,7 +9786,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="195" spans="1:3" ht="15">
+    <row r="195" spans="1:3">
       <c r="A195" s="36" t="s">
         <v>810</v>
       </c>
@@ -9791,7 +9797,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="196" spans="1:3" ht="15">
+    <row r="196" spans="1:3">
       <c r="A196" s="36" t="s">
         <v>810</v>
       </c>
@@ -9802,7 +9808,7 @@
         <v>824</v>
       </c>
     </row>
-    <row r="197" spans="1:3" ht="15">
+    <row r="197" spans="1:3">
       <c r="A197" s="39" t="s">
         <v>810</v>
       </c>
@@ -9821,7 +9827,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="56" customWidth="1"/>
@@ -9844,7 +9850,7 @@
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
     </row>
-    <row r="2" spans="1:11" ht="15">
+    <row r="2" spans="1:11">
       <c r="A2" s="36" t="s">
         <v>827</v>
       </c>
@@ -9852,7 +9858,7 @@
         <v>828</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="15">
+    <row r="3" spans="1:11">
       <c r="A3" s="36" t="s">
         <v>829</v>
       </c>
@@ -9860,7 +9866,7 @@
         <v>830</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="15">
+    <row r="4" spans="1:11">
       <c r="A4" s="36" t="s">
         <v>831</v>
       </c>
@@ -9868,7 +9874,7 @@
         <v>832</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="15">
+    <row r="5" spans="1:11">
       <c r="A5" s="36" t="s">
         <v>833</v>
       </c>
@@ -9876,7 +9882,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="15">
+    <row r="6" spans="1:11">
       <c r="A6" s="36" t="s">
         <v>835</v>
       </c>
@@ -9884,7 +9890,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="15">
+    <row r="7" spans="1:11">
       <c r="A7" s="39" t="s">
         <v>836</v>
       </c>
@@ -9900,7 +9906,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:K82"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="24" customWidth="1"/>
     <col min="3" max="4" width="18" customWidth="1"/>
@@ -11807,7 +11813,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:K25"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="120" customWidth="1"/>
   </cols>

</xml_diff>